<commit_message>
fix: a  major update
</commit_message>
<xml_diff>
--- a/data/sce_compartment_curation/2026_curated/fungal_type_cell_wall_annotations.xlsx
+++ b/data/sce_compartment_curation/2026_curated/fungal_type_cell_wall_annotations.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M107"/>
+  <dimension ref="A1:M104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2383,16 +2383,16 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>TDH3</t>
+          <t>SCW4</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>YGR192C</t>
+          <t>YGR279C</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2438,13 +2438,13 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>Delgado ML, et al. (2001) PMID:11158358</t>
+          <t>Cappellaro C, et al. (1998) PMID:9748433</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2499,22 +2499,22 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>Cappellaro C, et al. (1998) PMID:9748433</t>
+          <t>Yin QY, et al. (2005) PMID:15781460</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>SCW4</t>
+          <t>BGL2</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>YGR279C</t>
+          <t>YGR282C</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2560,13 +2560,13 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>Yin QY, et al. (2005) PMID:15781460</t>
+          <t>Cappellaro C, et al. (1998) PMID:9748433</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -2621,22 +2621,22 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>Cappellaro C, et al. (1998) PMID:9748433</t>
+          <t>Klebl F and Tanner W (1989) PMID:2509432</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>BGL2</t>
+          <t>DSE2</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>YGR282C</t>
+          <t>YHR143W</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2682,22 +2682,22 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>Klebl F and Tanner W (1989) PMID:2509432</t>
+          <t>Doolin MT, et al. (2001) PMID:11309124</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>DSE2</t>
+          <t>FLO5</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>YHR143W</t>
+          <t>YHR211W</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2743,22 +2743,22 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>Doolin MT, et al. (2001) PMID:11309124</t>
+          <t>Bony M, et al. (1998) PMID:9483793</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>FLO5</t>
+          <t>TIR3</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>YHR211W</t>
+          <t>YIL011W</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2804,22 +2804,22 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>Bony M, et al. (1998) PMID:9483793</t>
+          <t>Hamada K, et al. (1999) PMID:10383953</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>TIR3</t>
+          <t>BAR1</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>YIL011W</t>
+          <t>YIL015W</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2860,27 +2860,27 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2013-08-07</t>
+          <t>2017-03-08</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>Hamada K, et al. (1999) PMID:10383953</t>
+          <t>Moukadiri I, et al. (1999) PMID:10438739</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>BAR1</t>
+          <t>SIM1</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>YIL015W</t>
+          <t>YIL123W</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2921,27 +2921,27 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2017-03-08</t>
+          <t>2013-08-07</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>Moukadiri I, et al. (1999) PMID:10438739</t>
+          <t>Velours G, et al. (2002) PMID:11958935</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SIM1</t>
+          <t>YPS6</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>YIL123W</t>
+          <t>YIR039C</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2987,22 +2987,22 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>Velours G, et al. (2002) PMID:11958935</t>
+          <t>Hamada K, et al. (1999) PMID:10383953</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>YPS6</t>
+          <t>PRY3</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>YIR039C</t>
+          <t>YJL078C</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -3043,27 +3043,27 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2013-08-07</t>
+          <t>2021-07-29</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>Hamada K, et al. (1999) PMID:10383953</t>
+          <t>Cottier S, et al. (2020) PMID:32554483</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>TDH1</t>
+          <t>PRY3</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>YJL052W</t>
+          <t>YJL078C</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -3104,18 +3104,18 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2017-03-17</t>
+          <t>2013-08-07</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>Delgado ML, et al. (2001) PMID:11158358</t>
+          <t>Hamada K, et al. (1999) PMID:10383953</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -3165,27 +3165,27 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2021-07-29</t>
+          <t>2013-08-07</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>Cottier S, et al. (2020) PMID:32554483</t>
+          <t>Yin QY, et al. (2005) PMID:15781460</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>PRY3</t>
+          <t>CIS3</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>YJL078C</t>
+          <t>YJL158C</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -3231,22 +3231,22 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>Hamada K, et al. (1999) PMID:10383953</t>
+          <t>Yin QY, et al. (2005) PMID:15781460</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>PRY3</t>
+          <t>CIS3</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>YJL078C</t>
+          <t>YJL158C</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -3292,22 +3292,22 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>Yin QY, et al. (2005) PMID:15781460</t>
+          <t>Moukadiri I, et al. (1999) PMID:10438739</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>CIS3</t>
+          <t>HSP150</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>YJL158C</t>
+          <t>YJL159W</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -3353,22 +3353,22 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>Yin QY, et al. (2005) PMID:15781460</t>
+          <t>Kapteyn JC, et al. (1999) PMID:10209754</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>CIS3</t>
+          <t>HSP150</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>YJL158C</t>
+          <t>YJL159W</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3414,13 +3414,13 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>Moukadiri I, et al. (1999) PMID:10438739</t>
+          <t>Yun DJ, et al. (1997) PMID:9192695</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -3475,22 +3475,22 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>Kapteyn JC, et al. (1999) PMID:10209754</t>
+          <t>Yin QY, et al. (2005) PMID:15781460</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>HSP150</t>
+          <t>TOH1</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>YJL159W</t>
+          <t>YJL171C</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3536,22 +3536,22 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>Yun DJ, et al. (1997) PMID:9192695</t>
+          <t>Hamada K, et al. (1999) PMID:10383953</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>HSP150</t>
+          <t>SAG1</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>YJL159W</t>
+          <t>YJR004C</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -3597,22 +3597,22 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>Yin QY, et al. (2005) PMID:15781460</t>
+          <t>Hamada K, et al. (1999) PMID:10383953</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>TOH1</t>
+          <t>JSN1</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>YJL171C</t>
+          <t>YJR091C</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -3653,27 +3653,27 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>2013-08-07</t>
+          <t>2016-01-07</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>Hamada K, et al. (1999) PMID:10383953</t>
+          <t>Mitchell SF, et al. (2013) PMID:23222640</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>SAG1</t>
+          <t>DAN1</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>YJR004C</t>
+          <t>YJR150C</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -3719,22 +3719,22 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>Hamada K, et al. (1999) PMID:10383953</t>
+          <t>Mrsa V, et al. (1999) PMID:10322008</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>TDH2</t>
+          <t>DAN4</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>YJR009C</t>
+          <t>YJR151C</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -3780,22 +3780,22 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>Delgado ML, et al. (2001) PMID:11158358</t>
+          <t>Hamada K, et al. (1999) PMID:10383953</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>JSN1</t>
+          <t>CWP1</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>YJR091C</t>
+          <t>YKL096W</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -3836,27 +3836,27 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>2016-01-07</t>
+          <t>2013-08-07</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>Mitchell SF, et al. (2013) PMID:23222640</t>
+          <t>Yin QY, et al. (2005) PMID:15781460</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>DAN1</t>
+          <t>CWP1</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>YJR150C</t>
+          <t>YKL096W</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -3902,22 +3902,22 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>Mrsa V, et al. (1999) PMID:10322008</t>
+          <t>Kapteyn JC, et al. (1997) PMID:9335273</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>DAN4</t>
+          <t>CWP2</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>YJR151C</t>
+          <t>YKL096W-A</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -3963,22 +3963,22 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>Hamada K, et al. (1999) PMID:10383953</t>
+          <t>Breinig F and Schmitt MJ (2002) PMID:11956747</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>CWP1</t>
+          <t>PIR3</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>YKL096W</t>
+          <t>YKL163W</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -4024,22 +4024,22 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>Yin QY, et al. (2005) PMID:15781460</t>
+          <t>Yun DJ, et al. (1997) PMID:9192695</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>CWP1</t>
+          <t>PIR3</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>YKL096W</t>
+          <t>YKL163W</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -4085,22 +4085,22 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>Kapteyn JC, et al. (1997) PMID:9335273</t>
+          <t>Yin QY, et al. (2005) PMID:15781460</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>CWP2</t>
+          <t>PIR1</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>YKL096W-A</t>
+          <t>YKL164C</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -4146,22 +4146,22 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>Breinig F and Schmitt MJ (2002) PMID:11956747</t>
+          <t>Yun DJ, et al. (1997) PMID:9192695</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>PIR3</t>
+          <t>PIR1</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>YKL163W</t>
+          <t>YKL164C</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -4207,22 +4207,22 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>Yun DJ, et al. (1997) PMID:9192695</t>
+          <t>Yin QY, et al. (2005) PMID:15781460</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>PIR3</t>
+          <t>MCD4</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>YKL163W</t>
+          <t>YKL165C</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -4268,22 +4268,22 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>Yin QY, et al. (2005) PMID:15781460</t>
+          <t>Kalebina TS, et al. (2002) PMID:12023081</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>PIR1</t>
+          <t>FLO10</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>YKL164C</t>
+          <t>YKR102W</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -4309,7 +4309,7 @@
       <c r="H64" t="inlineStr"/>
       <c r="I64" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>ISS with FLO1</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
@@ -4324,27 +4324,27 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>2013-08-07</t>
+          <t>2014-10-02</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>Yun DJ, et al. (1997) PMID:9192695</t>
+          <t>Teunissen AW and Steensma HY (1995) PMID:7502576</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>PIR1</t>
+          <t>SSA2</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>YKL164C</t>
+          <t>YLL024C</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -4390,22 +4390,22 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>Yin QY, et al. (2005) PMID:15781460</t>
+          <t>López-Ribot JL and Chaffin WL (1996) PMID:8755907</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MCD4</t>
+          <t>AFB1</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>YKL165C</t>
+          <t>YLR040C</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -4451,22 +4451,22 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>Kalebina TS, et al. (2002) PMID:12023081</t>
+          <t>Hamada K, et al. (1999) PMID:10383953</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>FLO10</t>
+          <t>NFG1</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>YKR102W</t>
+          <t>YLR042C</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -4492,7 +4492,7 @@
       <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
         <is>
-          <t>ISS with FLO1</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
@@ -4507,27 +4507,27 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>2014-10-02</t>
+          <t>2013-08-07</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>Teunissen AW and Steensma HY (1995) PMID:7502576</t>
+          <t>Hamada K, et al. (1999) PMID:10383953</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>SSA2</t>
+          <t>NCW2</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>YLL024C</t>
+          <t>YLR194C</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -4573,22 +4573,22 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>López-Ribot JL and Chaffin WL (1996) PMID:8755907</t>
+          <t>Hamada K, et al. (1999) PMID:10383953</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>AFB1</t>
+          <t>CTS1</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>YLR040C</t>
+          <t>YLR286C</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -4634,22 +4634,22 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>Hamada K, et al. (1999) PMID:10383953</t>
+          <t>Kuranda MJ and Robbins PW (1991) PMID:1918080</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>NFG1</t>
+          <t>CTS1</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>YLR042C</t>
+          <t>YLR286C</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -4695,22 +4695,22 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>Hamada K, et al. (1999) PMID:10383953</t>
+          <t>Colman-Lerner A, et al. (2001) PMID:11747810</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>NCW2</t>
+          <t>EXG1</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>YLR194C</t>
+          <t>YLR300W</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -4756,22 +4756,22 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>Hamada K, et al. (1999) PMID:10383953</t>
+          <t>Cappellaro C, et al. (1998) PMID:9748433</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>CTS1</t>
+          <t>CCW14</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>YLR286C</t>
+          <t>YLR390W-A</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -4817,22 +4817,22 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>Kuranda MJ and Robbins PW (1991) PMID:1918080</t>
+          <t>Moukadiri I, et al. (1997) PMID:9079899</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>CTS1</t>
+          <t>CCW14</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>YLR286C</t>
+          <t>YLR390W-A</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -4878,22 +4878,22 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>Colman-Lerner A, et al. (2001) PMID:11747810</t>
+          <t>Mrsă V, et al. (1997) PMID:9301021</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>EXG1</t>
+          <t>CCW14</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>YLR300W</t>
+          <t>YLR390W-A</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -4939,22 +4939,22 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>Cappellaro C, et al. (1998) PMID:9748433</t>
+          <t>Yin QY, et al. (2005) PMID:15781460</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>CCW14</t>
+          <t>PLB2</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>YLR390W-A</t>
+          <t>YMR006C</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -5000,22 +5000,22 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>Moukadiri I, et al. (1997) PMID:9079899</t>
+          <t>Hamada K, et al. (1999) PMID:10383953</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>CCW14</t>
+          <t>PLB2</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>YLR390W-A</t>
+          <t>YMR006C</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -5061,22 +5061,22 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>Mrsă V, et al. (1997) PMID:9301021</t>
+          <t>Yin QY, et al. (2005) PMID:15781460</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>CCW14</t>
+          <t>GAS3</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>YLR390W-A</t>
+          <t>YMR215W</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -5128,16 +5128,16 @@
     </row>
     <row r="78">
       <c r="A78" s="1" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>PLB2</t>
+          <t>GAS3</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>YMR006C</t>
+          <t>YMR215W</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -5189,16 +5189,16 @@
     </row>
     <row r="79">
       <c r="A79" s="1" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>PLB2</t>
+          <t>SCW10</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>YMR006C</t>
+          <t>YMR305C</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -5250,16 +5250,16 @@
     </row>
     <row r="80">
       <c r="A80" s="1" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>GAS3</t>
+          <t>SCW10</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>YMR215W</t>
+          <t>YMR305C</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -5305,22 +5305,22 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>Yin QY, et al. (2005) PMID:15781460</t>
+          <t>Cappellaro C, et al. (1998) PMID:9748433</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>GAS3</t>
+          <t>GAS1</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>YMR215W</t>
+          <t>YMR307W</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -5366,22 +5366,22 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>Hamada K, et al. (1999) PMID:10383953</t>
+          <t>Yin QY, et al. (2005) PMID:15781460</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="n">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>SCW10</t>
+          <t>GAS1</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>YMR305C</t>
+          <t>YMR307W</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -5427,22 +5427,22 @@
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t>Yin QY, et al. (2005) PMID:15781460</t>
+          <t>Rolli E, et al. (2009) PMID:19793924</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>SCW10</t>
+          <t>SUN4</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>YMR305C</t>
+          <t>YNL066W</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -5488,22 +5488,22 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>Cappellaro C, et al. (1998) PMID:9748433</t>
+          <t>Velours G, et al. (2002) PMID:11958935</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>GAS1</t>
+          <t>YNL190W</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>YMR307W</t>
+          <t>YNL190W</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -5549,22 +5549,22 @@
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>Yin QY, et al. (2005) PMID:15781460</t>
+          <t>Hamada K, et al. (1999) PMID:10383953</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="n">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>GAS1</t>
+          <t>TOS6</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>YMR307W</t>
+          <t>YNL300W</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -5610,22 +5610,22 @@
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>Rolli E, et al. (2009) PMID:19793924</t>
+          <t>Hamada K, et al. (1999) PMID:10383953</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="n">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>SUN4</t>
+          <t>KRE1</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>YNL066W</t>
+          <t>YNL322C</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -5671,22 +5671,22 @@
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>Velours G, et al. (2002) PMID:11958935</t>
+          <t>Breinig F and Schmitt MJ (2002) PMID:11956747</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="n">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>YNL190W</t>
+          <t>EGT2</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>YNL190W</t>
+          <t>YNL327W</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -5738,16 +5738,16 @@
     </row>
     <row r="88">
       <c r="A88" s="1" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>TOS6</t>
+          <t>AGA1</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>YNL300W</t>
+          <t>YNR044W</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -5793,22 +5793,22 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>Hamada K, et al. (1999) PMID:10383953</t>
+          <t>Roy A, et al. (1991) PMID:2072914</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>KRE1</t>
+          <t>AGA1</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>YNL322C</t>
+          <t>YNR044W</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -5854,22 +5854,22 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>Breinig F and Schmitt MJ (2002) PMID:11956747</t>
+          <t>Cappellaro C, et al. (1994) PMID:7957044</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="n">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>EGT2</t>
+          <t>DSE4</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>YNL327W</t>
+          <t>YNR067C</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -5915,22 +5915,22 @@
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t>Hamada K, et al. (1999) PMID:10383953</t>
+          <t>Terashima H, et al. (2002) PMID:11935221</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>AGA1</t>
+          <t>GAS5</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>YNR044W</t>
+          <t>YOL030W</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -5976,22 +5976,22 @@
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t>Roy A, et al. (1991) PMID:2072914</t>
+          <t>Yin QY, et al. (2005) PMID:15781460</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="n">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>AGA1</t>
+          <t>GAS5</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>YNR044W</t>
+          <t>YOL030W</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -6037,22 +6037,22 @@
       </c>
       <c r="M92" t="inlineStr">
         <is>
-          <t>Cappellaro C, et al. (1994) PMID:7957044</t>
+          <t>Hamada K, et al. (1999) PMID:10383953</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>DSE4</t>
+          <t>GAS4</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>YNR067C</t>
+          <t>YOL132W</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -6098,22 +6098,22 @@
       </c>
       <c r="M93" t="inlineStr">
         <is>
-          <t>Terashima H, et al. (2002) PMID:11935221</t>
+          <t>Hamada K, et al. (1999) PMID:10383953</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>GAS5</t>
+          <t>ZPS1</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>YOL030W</t>
+          <t>YOL154W</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -6159,22 +6159,22 @@
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>Yin QY, et al. (2005) PMID:15781460</t>
+          <t>Terashima H, et al. (2002) PMID:11935221</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="n">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>GAS5</t>
+          <t>HPF1</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>YOL030W</t>
+          <t>YOL155C</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -6220,22 +6220,22 @@
       </c>
       <c r="M95" t="inlineStr">
         <is>
-          <t>Hamada K, et al. (1999) PMID:10383953</t>
+          <t>Horie T and Isono K (2001) PMID:11748726</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="n">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>GAS4</t>
+          <t>TIR4</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>YOL132W</t>
+          <t>YOR009W</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -6287,16 +6287,16 @@
     </row>
     <row r="97">
       <c r="A97" s="1" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>ZPS1</t>
+          <t>SPR1</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>YOL154W</t>
+          <t>YOR190W</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -6322,7 +6322,7 @@
       <c r="H97" t="inlineStr"/>
       <c r="I97" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>IMP</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
@@ -6342,22 +6342,22 @@
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>Terashima H, et al. (2002) PMID:11935221</t>
+          <t>Muthukumar G, et al. (1993) PMID:8419289</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>HPF1</t>
+          <t>SPR2</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>YOL155C</t>
+          <t>YOR214C</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -6403,22 +6403,22 @@
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>Horie T and Isono K (2001) PMID:11748726</t>
+          <t>Hamada K, et al. (1999) PMID:10383953</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>TIR4</t>
+          <t>SRL1</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>YOR009W</t>
+          <t>YOR247W</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -6464,22 +6464,22 @@
       </c>
       <c r="M99" t="inlineStr">
         <is>
-          <t>Hamada K, et al. (1999) PMID:10383953</t>
+          <t>Terashima H, et al. (2002) PMID:11935221</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="n">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>SPR1</t>
+          <t>FIT2</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>YOR190W</t>
+          <t>YOR382W</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -6505,7 +6505,7 @@
       <c r="H100" t="inlineStr"/>
       <c r="I100" t="inlineStr">
         <is>
-          <t>IMP</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
@@ -6525,22 +6525,22 @@
       </c>
       <c r="M100" t="inlineStr">
         <is>
-          <t>Muthukumar G, et al. (1993) PMID:8419289</t>
+          <t>Hamada K, et al. (1999) PMID:10383953</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="n">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>SPR2</t>
+          <t>FIT3</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>YOR214C</t>
+          <t>YOR383C</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -6592,16 +6592,16 @@
     </row>
     <row r="102">
       <c r="A102" s="1" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>SRL1</t>
+          <t>SPO19</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>YOR247W</t>
+          <t>YPL130W</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -6647,22 +6647,22 @@
       </c>
       <c r="M102" t="inlineStr">
         <is>
-          <t>Terashima H, et al. (2002) PMID:11935221</t>
+          <t>Hamada K, et al. (1999) PMID:10383953</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>FIT2</t>
+          <t>SVS1</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>YOR382W</t>
+          <t>YPL163C</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -6708,22 +6708,22 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>Hamada K, et al. (1999) PMID:10383953</t>
+          <t>Terashima H, et al. (2002) PMID:11935221</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="1" t="n">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>FIT3</t>
+          <t>ATH1</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>YOR383C</t>
+          <t>YPR026W</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -6768,189 +6768,6 @@
         </is>
       </c>
       <c r="M104" t="inlineStr">
-        <is>
-          <t>Hamada K, et al. (1999) PMID:10383953</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="1" t="n">
-        <v>108</v>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>SPO19</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>YPL130W</t>
-        </is>
-      </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>located in</t>
-        </is>
-      </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>GO:0009277</t>
-        </is>
-      </c>
-      <c r="F105" t="inlineStr">
-        <is>
-          <t>fungal-type cell wall</t>
-        </is>
-      </c>
-      <c r="G105" t="inlineStr">
-        <is>
-          <t>cellular component</t>
-        </is>
-      </c>
-      <c r="H105" t="inlineStr"/>
-      <c r="I105" t="inlineStr">
-        <is>
-          <t>IDA</t>
-        </is>
-      </c>
-      <c r="J105" t="inlineStr">
-        <is>
-          <t>manually curated</t>
-        </is>
-      </c>
-      <c r="K105" t="inlineStr">
-        <is>
-          <t>SGD</t>
-        </is>
-      </c>
-      <c r="L105" t="inlineStr">
-        <is>
-          <t>2013-08-07</t>
-        </is>
-      </c>
-      <c r="M105" t="inlineStr">
-        <is>
-          <t>Hamada K, et al. (1999) PMID:10383953</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="1" t="n">
-        <v>109</v>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>SVS1</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>YPL163C</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr">
-        <is>
-          <t>located in</t>
-        </is>
-      </c>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>GO:0009277</t>
-        </is>
-      </c>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t>fungal-type cell wall</t>
-        </is>
-      </c>
-      <c r="G106" t="inlineStr">
-        <is>
-          <t>cellular component</t>
-        </is>
-      </c>
-      <c r="H106" t="inlineStr"/>
-      <c r="I106" t="inlineStr">
-        <is>
-          <t>IDA</t>
-        </is>
-      </c>
-      <c r="J106" t="inlineStr">
-        <is>
-          <t>manually curated</t>
-        </is>
-      </c>
-      <c r="K106" t="inlineStr">
-        <is>
-          <t>SGD</t>
-        </is>
-      </c>
-      <c r="L106" t="inlineStr">
-        <is>
-          <t>2013-08-07</t>
-        </is>
-      </c>
-      <c r="M106" t="inlineStr">
-        <is>
-          <t>Terashima H, et al. (2002) PMID:11935221</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="1" t="n">
-        <v>110</v>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>ATH1</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>YPR026W</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>located in</t>
-        </is>
-      </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>GO:0009277</t>
-        </is>
-      </c>
-      <c r="F107" t="inlineStr">
-        <is>
-          <t>fungal-type cell wall</t>
-        </is>
-      </c>
-      <c r="G107" t="inlineStr">
-        <is>
-          <t>cellular component</t>
-        </is>
-      </c>
-      <c r="H107" t="inlineStr"/>
-      <c r="I107" t="inlineStr">
-        <is>
-          <t>IDA</t>
-        </is>
-      </c>
-      <c r="J107" t="inlineStr">
-        <is>
-          <t>manually curated</t>
-        </is>
-      </c>
-      <c r="K107" t="inlineStr">
-        <is>
-          <t>SGD</t>
-        </is>
-      </c>
-      <c r="L107" t="inlineStr">
-        <is>
-          <t>2013-08-07</t>
-        </is>
-      </c>
-      <c r="M107" t="inlineStr">
         <is>
           <t>Jules M, et al. (2004) PMID:15128531</t>
         </is>

</xml_diff>